<commit_message>
FIXED: price in tables
</commit_message>
<xml_diff>
--- a/media/price_lists/fijamom.xlsx
+++ b/media/price_lists/fijamom.xlsx
@@ -505,8 +505,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>950.0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1178.00</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -543,8 +551,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1870.0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2318.80</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -581,8 +597,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1050.0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1302.00</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -619,8 +643,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1488.00</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -657,8 +689,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>132.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>163.68</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -695,8 +735,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>138.88</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -733,8 +781,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>880.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1091.20</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -771,8 +827,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2674.0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>3315.76</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -809,8 +873,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>275.0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>341.00</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -847,8 +919,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>586.0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>726.64</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -885,8 +965,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>758.0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>939.92</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -923,8 +1011,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>887.0</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1099.88</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -961,8 +1057,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1058.0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1311.92</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -999,8 +1103,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2860.0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>3546.40</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1037,8 +1149,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>400.0</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>496.00</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1075,8 +1195,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>429.0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>531.96</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1113,8 +1241,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2548.0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>3159.52</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1151,8 +1287,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3350.0</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>4154.00</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1189,8 +1333,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3960.0</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>4910.40</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1227,8 +1379,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>5656.0</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>7013.44</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1265,8 +1425,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>8437.0</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>10461.88</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1303,8 +1471,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10439.0</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>12944.36</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1341,8 +1517,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>14729.0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>18263.96</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1379,8 +1563,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>16159.0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>20037.16</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1417,8 +1609,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>18590.0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>23051.60</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1455,8 +1655,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>20020.0</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>24824.80</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1493,8 +1701,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>19800.0</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>24552.00</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1531,8 +1747,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1400.0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1736.00</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1569,8 +1793,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>1144.0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>1418.56</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1607,8 +1839,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>550.0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>682.00</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1645,8 +1885,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>1430.0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1773.20</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1683,8 +1931,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>308.0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>381.92</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1721,8 +1977,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>1045.0</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>1295.80</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1759,8 +2023,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>6435.0</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>7979.40</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1797,8 +2069,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>3960.0</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>4910.40</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1835,8 +2115,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1859.0</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2305.16</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1873,8 +2161,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>1859.0</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2305.16</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1911,8 +2207,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>1859.0</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2305.16</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1949,8 +2253,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2288.0</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2837.12</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -1987,8 +2299,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2288.0</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2837.12</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2025,8 +2345,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2288.0</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2837.12</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2063,8 +2391,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>3289.0</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>4078.36</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2101,8 +2437,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>3718.0</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>4610.32</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2139,8 +2483,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>3718.0</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>4610.32</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2177,8 +2529,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>1573.0</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>1950.52</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2215,8 +2575,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>660.0</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>818.40</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2253,8 +2621,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>990.0</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>1227.60</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2291,8 +2667,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>275.0</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>341.00</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2329,8 +2713,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>16.12</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2367,8 +2759,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>12870.0</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>15958.80</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2405,8 +2805,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>132.0</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>163.68</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2443,8 +2851,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>132.0</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>163.68</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2481,8 +2897,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>132.0</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>163.68</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2519,8 +2943,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>264.0</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>327.36</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2557,8 +2989,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>11000.0</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>13640.00</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2595,8 +3035,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>8075.0</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>10013.00</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2633,8 +3081,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>9922.0</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>12303.28</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2671,8 +3127,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>1316.0</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>1631.84</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2709,8 +3173,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2002.0</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2482.48</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2747,8 +3219,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2116.0</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2623.84</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2785,8 +3265,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>3375.0</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>4185.00</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2823,8 +3311,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>1430.0</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>1773.20</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2861,8 +3357,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>110000.0</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>136400.00</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2899,8 +3403,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>110000.0</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>136400.00</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2937,8 +3449,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>38500.0</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>47740.00</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -2975,8 +3495,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>12100.0</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>15004.00</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3013,8 +3541,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>6000.0</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>7440.00</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3051,8 +3587,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>15000.0</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>18600.00</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3089,8 +3633,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>1364.00</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3127,8 +3679,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>3500.0</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>4340.00</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3165,8 +3725,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>250000.0</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>310000.00</t>
+        </is>
+      </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3203,8 +3771,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>7000.0</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>8680.00</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3241,8 +3817,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>2480.00</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3279,8 +3863,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>20000.0</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>24800.00</t>
+        </is>
+      </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3317,8 +3909,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>9920.00</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3355,8 +3955,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>3100.00</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3393,8 +4001,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>8500.0</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>10540.00</t>
+        </is>
+      </c>
       <c r="I78" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3431,8 +4047,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>30000.0</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>37200.00</t>
+        </is>
+      </c>
       <c r="I79" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3469,8 +4093,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>40000.0</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>49600.00</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3507,8 +4139,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>1240.00</t>
+        </is>
+      </c>
       <c r="I81" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3545,8 +4185,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>50000.0</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>62000.00</t>
+        </is>
+      </c>
       <c r="I82" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3583,8 +4231,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>65000.0</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>80600.00</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3621,8 +4277,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>20000.0</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>24800.00</t>
+        </is>
+      </c>
       <c r="I84" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3659,8 +4323,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>400000.0</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>496000.00</t>
+        </is>
+      </c>
       <c r="I85" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3697,8 +4369,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>76000.0</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>94240.00</t>
+        </is>
+      </c>
       <c r="I86" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3735,8 +4415,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>320000.0</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>396800.00</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3773,8 +4461,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>79200.0</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>98208.00</t>
+        </is>
+      </c>
       <c r="I88" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3811,8 +4507,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>280000.0</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>347200.00</t>
+        </is>
+      </c>
       <c r="I89" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3849,8 +4553,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>643500.0</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>797940.00</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3887,8 +4599,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>643500.0</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>797940.00</t>
+        </is>
+      </c>
       <c r="I91" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3925,8 +4645,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>643500.0</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>797940.00</t>
+        </is>
+      </c>
       <c r="I92" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -3963,8 +4691,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>643500.0</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>797940.00</t>
+        </is>
+      </c>
       <c r="I93" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4001,8 +4737,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>643500.0</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>797940.00</t>
+        </is>
+      </c>
       <c r="I94" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4039,8 +4783,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>759330.0</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>941569.20</t>
+        </is>
+      </c>
       <c r="I95" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4077,8 +4829,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>707850.0</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>877734.00</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4115,8 +4875,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>965250.0</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>1196910.00</t>
+        </is>
+      </c>
       <c r="I97" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4153,8 +4921,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2574000.0</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>3191760.00</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4191,8 +4967,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2059200.0</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2553408.00</t>
+        </is>
+      </c>
       <c r="I99" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4229,8 +5013,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2574000.0</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>3191760.00</t>
+        </is>
+      </c>
       <c r="I100" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4267,8 +5059,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>836550.0</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>1037322.00</t>
+        </is>
+      </c>
       <c r="I101" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4305,8 +5105,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>965250.0</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>1196910.00</t>
+        </is>
+      </c>
       <c r="I102" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4343,8 +5151,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>1544400.0</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>1915056.00</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4381,8 +5197,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2187900.0</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>2712996.00</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4419,8 +5243,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>1784640.0</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>2212953.60</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4457,8 +5289,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2059200.0</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>2553408.00</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4495,8 +5335,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>3217500.0</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>3989700.00</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4533,8 +5381,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2123550.0</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2633202.00</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4571,8 +5427,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>3861000.0</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>4787640.00</t>
+        </is>
+      </c>
       <c r="I109" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4609,8 +5473,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2895750.0</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>3590730.00</t>
+        </is>
+      </c>
       <c r="I110" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4647,8 +5519,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>3377660.0</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>4188298.40</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4685,8 +5565,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>4979260.0</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>6174282.40</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4723,8 +5611,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>1673100.0</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2074644.00</t>
+        </is>
+      </c>
       <c r="I113" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4761,8 +5657,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>939510.0</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>1164992.40</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4799,8 +5703,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>1158300.0</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>1436292.00</t>
+        </is>
+      </c>
       <c r="I115" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4837,8 +5749,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>3603600.0</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>4468464.00</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4875,8 +5795,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>3732300.0</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>4628052.00</t>
+        </is>
+      </c>
       <c r="I117" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4913,8 +5841,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>1132560.0</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>1404374.40</t>
+        </is>
+      </c>
       <c r="I118" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4951,8 +5887,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>1158300.0</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>1436292.00</t>
+        </is>
+      </c>
       <c r="I119" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -4989,8 +5933,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>1415700.0</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>1755468.00</t>
+        </is>
+      </c>
       <c r="I120" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -5027,8 +5979,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>1847560.0</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2290974.40</t>
+        </is>
+      </c>
       <c r="I121" t="inlineStr">
         <is>
           <t>skipped</t>
@@ -5065,8 +6025,16 @@
           <t>1400.0</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>1850.0</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2294.00</t>
+        </is>
+      </c>
       <c r="I122" t="inlineStr">
         <is>
           <t>skipped</t>

</xml_diff>